<commit_message>
Adiciona Docker, identificacao por patrimonio/descricao e licenca MIT
- docker-compose.yml + Dockerfiles + nginx.conf (deploy completo)
- Excel: reconhece coluna de patrimonio/inventario/tombamento e usa
  descricao como identificador quando nao ha codigo (nunca mais "Linha N")
- Busca/filtro por codigo, patrimonio ou descricao em Captura, Dashboard,
  Lista e Auditoria
- iniciar.bat autossuficiente (instala dependencias na primeira vez)
- LICENSE (MIT)
</commit_message>
<xml_diff>
--- a/backend/data/ativos_exemplo.xlsx
+++ b/backend/data/ativos_exemplo.xlsx
@@ -397,17 +397,18 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:I13"/>
+  <dimension ref="A1:J14"/>
   <cols>
     <col min="1" max="1" width="10.83203125" customWidth="1"/>
-    <col min="2" max="2" width="38.83203125" customWidth="1"/>
-    <col min="3" max="3" width="14.83203125" customWidth="1"/>
-    <col min="4" max="4" width="20.83203125" customWidth="1"/>
-    <col min="5" max="5" width="10.83203125" customWidth="1"/>
-    <col min="6" max="6" width="8.83203125" customWidth="1"/>
-    <col min="7" max="7" width="18.83203125" customWidth="1"/>
-    <col min="8" max="8" width="7.83203125" customWidth="1"/>
-    <col min="9" max="9" width="28.83203125" customWidth="1"/>
+    <col min="2" max="2" width="12.83203125" customWidth="1"/>
+    <col min="3" max="3" width="38.83203125" customWidth="1"/>
+    <col min="4" max="4" width="14.83203125" customWidth="1"/>
+    <col min="5" max="5" width="20.83203125" customWidth="1"/>
+    <col min="6" max="6" width="10.83203125" customWidth="1"/>
+    <col min="7" max="7" width="8.83203125" customWidth="1"/>
+    <col min="8" max="8" width="18.83203125" customWidth="1"/>
+    <col min="9" max="9" width="7.83203125" customWidth="1"/>
+    <col min="10" max="10" width="28.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -415,27 +416,30 @@
         <v>Código</v>
       </c>
       <c r="B1" t="str">
+        <v>Patrimônio</v>
+      </c>
+      <c r="C1" t="str">
         <v>Descrição</v>
       </c>
-      <c r="C1" t="str">
+      <c r="D1" t="str">
         <v>Fabricante</v>
       </c>
-      <c r="D1" t="str">
+      <c r="E1" t="str">
         <v>Modelo</v>
       </c>
-      <c r="E1" t="str">
+      <c r="F1" t="str">
         <v>Potência</v>
       </c>
-      <c r="F1" t="str">
+      <c r="G1" t="str">
         <v>RPM</v>
       </c>
-      <c r="G1" t="str">
+      <c r="H1" t="str">
         <v>Voltagem</v>
       </c>
-      <c r="H1" t="str">
+      <c r="I1" t="str">
         <v>Ano</v>
       </c>
-      <c r="I1" t="str">
+      <c r="J1" t="str">
         <v>Localização Esperada</v>
       </c>
     </row>
@@ -444,27 +448,30 @@
         <v>MOT-001</v>
       </c>
       <c r="B2" t="str">
+        <v>2021.004512</v>
+      </c>
+      <c r="C2" t="str">
         <v>Motor elétrico de indução trifásico</v>
       </c>
-      <c r="C2" t="str">
+      <c r="D2" t="str">
         <v>WEG</v>
       </c>
-      <c r="D2" t="str">
+      <c r="E2" t="str">
         <v>W22 IR3 Premium</v>
       </c>
-      <c r="E2" t="str">
+      <c r="F2" t="str">
         <v>15 cv</v>
       </c>
-      <c r="F2" t="str">
+      <c r="G2" t="str">
         <v>3540</v>
       </c>
-      <c r="G2" t="str">
+      <c r="H2" t="str">
         <v>380/660 V</v>
       </c>
-      <c r="H2" t="str">
+      <c r="I2" t="str">
         <v>2016</v>
       </c>
-      <c r="I2" t="str">
+      <c r="J2" t="str">
         <v>Casa de Bombas - Nível 1</v>
       </c>
     </row>
@@ -473,27 +480,30 @@
         <v>MOT-002</v>
       </c>
       <c r="B3" t="str">
+        <v>2021.004513</v>
+      </c>
+      <c r="C3" t="str">
         <v>Motor elétrico de indução trifásico</v>
       </c>
-      <c r="C3" t="str">
+      <c r="D3" t="str">
         <v>WEG</v>
       </c>
-      <c r="D3" t="str">
+      <c r="E3" t="str">
         <v>W21</v>
       </c>
-      <c r="E3" t="str">
+      <c r="F3" t="str">
         <v>10 cv</v>
       </c>
-      <c r="F3" t="str">
+      <c r="G3" t="str">
         <v>1760</v>
       </c>
-      <c r="G3" t="str">
+      <c r="H3" t="str">
         <v>220/380 V</v>
       </c>
-      <c r="H3" t="str">
+      <c r="I3" t="str">
         <v>2012</v>
       </c>
-      <c r="I3" t="str">
+      <c r="J3" t="str">
         <v>Linha de Envase A</v>
       </c>
     </row>
@@ -502,27 +512,30 @@
         <v>MOT-003</v>
       </c>
       <c r="B4" t="str">
+        <v>2021.004514</v>
+      </c>
+      <c r="C4" t="str">
         <v>Motor elétrico alta rotação</v>
       </c>
-      <c r="C4" t="str">
+      <c r="D4" t="str">
         <v>Siemens</v>
       </c>
-      <c r="D4" t="str">
+      <c r="E4" t="str">
         <v>1LE0</v>
       </c>
-      <c r="E4" t="str">
+      <c r="F4" t="str">
         <v>20 cv</v>
       </c>
-      <c r="F4" t="str">
+      <c r="G4" t="str">
         <v>1780</v>
       </c>
-      <c r="G4" t="str">
+      <c r="H4" t="str">
         <v>380 V</v>
       </c>
-      <c r="H4" t="str">
+      <c r="I4" t="str">
         <v>2018</v>
       </c>
-      <c r="I4" t="str">
+      <c r="J4" t="str">
         <v>Torre de Resfriamento</v>
       </c>
     </row>
@@ -531,27 +544,30 @@
         <v>CMP-001</v>
       </c>
       <c r="B5" t="str">
+        <v>2019.001187</v>
+      </c>
+      <c r="C5" t="str">
         <v>Compressor de ar parafuso</v>
       </c>
-      <c r="C5" t="str">
+      <c r="D5" t="str">
         <v>Atlas Copco</v>
       </c>
-      <c r="D5" t="str">
+      <c r="E5" t="str">
         <v>GA 30</v>
       </c>
-      <c r="E5" t="str">
+      <c r="F5" t="str">
         <v>40 cv</v>
       </c>
-      <c r="F5" t="str">
+      <c r="G5" t="str">
         <v>2970</v>
       </c>
-      <c r="G5" t="str">
+      <c r="H5" t="str">
         <v>440 V</v>
       </c>
-      <c r="H5" t="str">
+      <c r="I5" t="str">
         <v>2010</v>
       </c>
-      <c r="I5" t="str">
+      <c r="J5" t="str">
         <v>Central de Ar Comprimido</v>
       </c>
     </row>
@@ -560,27 +576,30 @@
         <v>CMP-002</v>
       </c>
       <c r="B6" t="str">
+        <v>2019.001188</v>
+      </c>
+      <c r="C6" t="str">
         <v>Compressor de ar pistão</v>
       </c>
-      <c r="C6" t="str">
+      <c r="D6" t="str">
         <v>Schulz</v>
       </c>
-      <c r="D6" t="str">
+      <c r="E6" t="str">
         <v>MSV 40 MAX</v>
       </c>
-      <c r="E6" t="str">
+      <c r="F6" t="str">
         <v>10 cv</v>
       </c>
-      <c r="F6" t="str">
+      <c r="G6" t="str">
         <v>1150</v>
       </c>
-      <c r="G6" t="str">
+      <c r="H6" t="str">
         <v>220 V</v>
       </c>
-      <c r="H6" t="str">
+      <c r="I6" t="str">
         <v>2009</v>
       </c>
-      <c r="I6" t="str">
+      <c r="J6" t="str">
         <v>Oficina de Manutenção</v>
       </c>
     </row>
@@ -589,27 +608,30 @@
         <v>BMB-001</v>
       </c>
       <c r="B7" t="str">
+        <v>2020.002230</v>
+      </c>
+      <c r="C7" t="str">
         <v>Bomba centrífuga de recalque</v>
       </c>
-      <c r="C7" t="str">
+      <c r="D7" t="str">
         <v>KSB</v>
       </c>
-      <c r="D7" t="str">
+      <c r="E7" t="str">
         <v>Meganorm 50-160</v>
       </c>
-      <c r="E7" t="str">
+      <c r="F7" t="str">
         <v>7,5 cv</v>
       </c>
-      <c r="F7" t="str">
+      <c r="G7" t="str">
         <v>3480</v>
       </c>
-      <c r="G7" t="str">
+      <c r="H7" t="str">
         <v>380 V</v>
       </c>
-      <c r="H7" t="str">
+      <c r="I7" t="str">
         <v>2015</v>
       </c>
-      <c r="I7" t="str">
+      <c r="J7" t="str">
         <v>Casa de Bombas - Nível 2</v>
       </c>
     </row>
@@ -618,27 +640,30 @@
         <v>BMB-002</v>
       </c>
       <c r="B8" t="str">
+        <v>2020.002231</v>
+      </c>
+      <c r="C8" t="str">
         <v>Bomba centrífuga de processo</v>
       </c>
-      <c r="C8" t="str">
+      <c r="D8" t="str">
         <v>Grundfos</v>
       </c>
-      <c r="D8" t="str">
+      <c r="E8" t="str">
         <v>NB 65-200</v>
       </c>
-      <c r="E8" t="str">
+      <c r="F8" t="str">
         <v>25 cv</v>
       </c>
-      <c r="F8" t="str">
+      <c r="G8" t="str">
         <v>1750</v>
       </c>
-      <c r="G8" t="str">
+      <c r="H8" t="str">
         <v>440 V</v>
       </c>
-      <c r="H8" t="str">
+      <c r="I8" t="str">
         <v>2019</v>
       </c>
-      <c r="I8" t="str">
+      <c r="J8" t="str">
         <v>Sala de Processo B</v>
       </c>
     </row>
@@ -647,27 +672,30 @@
         <v>TRF-001</v>
       </c>
       <c r="B9" t="str">
+        <v>2011.000045</v>
+      </c>
+      <c r="C9" t="str">
         <v>Transformador a seco</v>
       </c>
-      <c r="C9" t="str">
+      <c r="D9" t="str">
         <v>ABB</v>
       </c>
-      <c r="D9" t="str">
+      <c r="E9" t="str">
         <v>RESIBLOC 750</v>
       </c>
-      <c r="E9" t="str">
+      <c r="F9" t="str">
         <v>750 kVA</v>
       </c>
-      <c r="F9" t="str">
+      <c r="G9" t="str">
         <v/>
       </c>
-      <c r="G9" t="str">
+      <c r="H9" t="str">
         <v>13,8 kV / 380 V</v>
       </c>
-      <c r="H9" t="str">
+      <c r="I9" t="str">
         <v>2011</v>
       </c>
-      <c r="I9" t="str">
+      <c r="J9" t="str">
         <v>Subestação Principal</v>
       </c>
     </row>
@@ -676,27 +704,30 @@
         <v>TRF-002</v>
       </c>
       <c r="B10" t="str">
+        <v>2008.000032</v>
+      </c>
+      <c r="C10" t="str">
         <v>Transformador óleo</v>
       </c>
-      <c r="C10" t="str">
+      <c r="D10" t="str">
         <v>WEG</v>
       </c>
-      <c r="D10" t="str">
+      <c r="E10" t="str">
         <v>TTD 300</v>
       </c>
-      <c r="E10" t="str">
+      <c r="F10" t="str">
         <v>300 kVA</v>
       </c>
-      <c r="F10" t="str">
+      <c r="G10" t="str">
         <v/>
       </c>
-      <c r="G10" t="str">
+      <c r="H10" t="str">
         <v>13,8 kV / 220 V</v>
       </c>
-      <c r="H10" t="str">
+      <c r="I10" t="str">
         <v>2008</v>
       </c>
-      <c r="I10" t="str">
+      <c r="J10" t="str">
         <v>Subestação Auxiliar</v>
       </c>
     </row>
@@ -705,45 +736,48 @@
         <v>VNT-001</v>
       </c>
       <c r="B11" t="str">
+        <v>2017.003301</v>
+      </c>
+      <c r="C11" t="str">
         <v>Ventilador industrial axial</v>
       </c>
-      <c r="C11" t="str">
+      <c r="D11" t="str">
         <v>Otam</v>
       </c>
-      <c r="D11" t="str">
+      <c r="E11" t="str">
         <v>AXN 900</v>
       </c>
-      <c r="E11" t="str">
+      <c r="F11" t="str">
         <v>30 cv</v>
       </c>
-      <c r="F11" t="str">
+      <c r="G11" t="str">
         <v>1170</v>
       </c>
-      <c r="G11" t="str">
+      <c r="H11" t="str">
         <v>380 V</v>
       </c>
-      <c r="H11" t="str">
+      <c r="I11" t="str">
         <v>2017</v>
       </c>
-      <c r="I11" t="str">
+      <c r="J11" t="str">
         <v>Exaustão Galpão 3</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="str">
-        <v>RED-001</v>
+        <v/>
       </c>
       <c r="B12" t="str">
+        <v>2014.001099</v>
+      </c>
+      <c r="C12" t="str">
         <v>Redutor de velocidade</v>
       </c>
-      <c r="C12" t="str">
+      <c r="D12" t="str">
         <v>SEW</v>
       </c>
-      <c r="D12" t="str">
+      <c r="E12" t="str">
         <v>R107</v>
-      </c>
-      <c r="E12" t="str">
-        <v>—</v>
       </c>
       <c r="F12" t="str">
         <v>—</v>
@@ -752,9 +786,12 @@
         <v>—</v>
       </c>
       <c r="H12" t="str">
+        <v>—</v>
+      </c>
+      <c r="I12" t="str">
         <v>2014</v>
       </c>
-      <c r="I12" t="str">
+      <c r="J12" t="str">
         <v>Transportador TC-05</v>
       </c>
     </row>
@@ -763,33 +800,68 @@
         <v>GER-001</v>
       </c>
       <c r="B13" t="str">
+        <v>2013.000871</v>
+      </c>
+      <c r="C13" t="str">
         <v>Grupo gerador diesel standby</v>
       </c>
-      <c r="C13" t="str">
+      <c r="D13" t="str">
         <v>Stemac</v>
       </c>
-      <c r="D13" t="str">
+      <c r="E13" t="str">
         <v>ST 250</v>
       </c>
-      <c r="E13" t="str">
+      <c r="F13" t="str">
         <v>250 kVA</v>
       </c>
-      <c r="F13" t="str">
+      <c r="G13" t="str">
         <v>1800</v>
       </c>
-      <c r="G13" t="str">
+      <c r="H13" t="str">
         <v>380 V</v>
       </c>
-      <c r="H13" t="str">
+      <c r="I13" t="str">
         <v>2013</v>
       </c>
-      <c r="I13" t="str">
+      <c r="J13" t="str">
         <v>Casa de Força</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="str">
+        <v/>
+      </c>
+      <c r="B14" t="str">
+        <v/>
+      </c>
+      <c r="C14" t="str">
+        <v>Painel elétrico de comando geral</v>
+      </c>
+      <c r="D14" t="str">
+        <v>WEG</v>
+      </c>
+      <c r="E14" t="str">
+        <v>—</v>
+      </c>
+      <c r="F14" t="str">
+        <v>—</v>
+      </c>
+      <c r="G14" t="str">
+        <v>—</v>
+      </c>
+      <c r="H14" t="str">
+        <v>380 V</v>
+      </c>
+      <c r="I14" t="str">
+        <v>2015</v>
+      </c>
+      <c r="J14" t="str">
+        <v>Sala de Painéis</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:I13"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:J14"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>